<commit_message>
Fix Rank formula to survive row sorting
The original formula in V<n> contained a hard-coded literal row number in
the tie-breaker — (ROW(U$3:U$32)<n) — so when rows are sorted in Excel,
the formula moves with its row but the literal n stays put. Each candidate's
tie-breaker then references a wrong row position, producing duplicate
ranks and a top rank that no longer starts at 1.

Replaced the literal with ROW(), which always evaluates to the current
cell's row. The rank now stays correct under any sort order.

Claude-Session: https://claude.ai/code/session_01RrRTkwXtHjLLkRsnwRC4Uu
</commit_message>
<xml_diff>
--- a/gnc_june_2026/gnc_intern_evaluation_v1.xlsx
+++ b/gnc_june_2026/gnc_intern_evaluation_v1.xlsx
@@ -2090,7 +2090,7 @@
         <v/>
       </c>
       <c r="V3" s="9">
-        <f>IF(OR(B3="",T3="Y"),"",1+SUMPRODUCT(((U$3:U$32&gt;U3)+((U$3:U$32=U3)*(ROW(U$3:U$32)&lt;3)))*(T$3:T$32&lt;&gt;"Y")*(B$3:B$32&lt;&gt;"")))</f>
+        <f>IF(OR(B3="",T3="Y"),"",1+SUMPRODUCT(((U$3:U$32&gt;U3)+((U$3:U$32=U3)*(ROW(U$3:U$32)&lt;ROW())))*(T$3:T$32&lt;&gt;"Y")*(B$3:B$32&lt;&gt;"")))</f>
         <v/>
       </c>
       <c r="W3" s="6" t="inlineStr">
@@ -2193,7 +2193,7 @@
         <v/>
       </c>
       <c r="V4" s="9">
-        <f>IF(OR(B4="",T4="Y"),"",1+SUMPRODUCT(((U$3:U$32&gt;U4)+((U$3:U$32=U4)*(ROW(U$3:U$32)&lt;4)))*(T$3:T$32&lt;&gt;"Y")*(B$3:B$32&lt;&gt;"")))</f>
+        <f>IF(OR(B4="",T4="Y"),"",1+SUMPRODUCT(((U$3:U$32&gt;U4)+((U$3:U$32=U4)*(ROW(U$3:U$32)&lt;ROW())))*(T$3:T$32&lt;&gt;"Y")*(B$3:B$32&lt;&gt;"")))</f>
         <v/>
       </c>
       <c r="W4" s="6" t="inlineStr">
@@ -2294,7 +2294,7 @@
         <v/>
       </c>
       <c r="V5" s="9">
-        <f>IF(OR(B5="",T5="Y"),"",1+SUMPRODUCT(((U$3:U$32&gt;U5)+((U$3:U$32=U5)*(ROW(U$3:U$32)&lt;5)))*(T$3:T$32&lt;&gt;"Y")*(B$3:B$32&lt;&gt;"")))</f>
+        <f>IF(OR(B5="",T5="Y"),"",1+SUMPRODUCT(((U$3:U$32&gt;U5)+((U$3:U$32=U5)*(ROW(U$3:U$32)&lt;ROW())))*(T$3:T$32&lt;&gt;"Y")*(B$3:B$32&lt;&gt;"")))</f>
         <v/>
       </c>
       <c r="W5" s="6" t="inlineStr">
@@ -2395,7 +2395,7 @@
         <v/>
       </c>
       <c r="V6" s="9">
-        <f>IF(OR(B6="",T6="Y"),"",1+SUMPRODUCT(((U$3:U$32&gt;U6)+((U$3:U$32=U6)*(ROW(U$3:U$32)&lt;6)))*(T$3:T$32&lt;&gt;"Y")*(B$3:B$32&lt;&gt;"")))</f>
+        <f>IF(OR(B6="",T6="Y"),"",1+SUMPRODUCT(((U$3:U$32&gt;U6)+((U$3:U$32=U6)*(ROW(U$3:U$32)&lt;ROW())))*(T$3:T$32&lt;&gt;"Y")*(B$3:B$32&lt;&gt;"")))</f>
         <v/>
       </c>
       <c r="W6" s="6" t="inlineStr">
@@ -2498,7 +2498,7 @@
         <v/>
       </c>
       <c r="V7" s="9">
-        <f>IF(OR(B7="",T7="Y"),"",1+SUMPRODUCT(((U$3:U$32&gt;U7)+((U$3:U$32=U7)*(ROW(U$3:U$32)&lt;7)))*(T$3:T$32&lt;&gt;"Y")*(B$3:B$32&lt;&gt;"")))</f>
+        <f>IF(OR(B7="",T7="Y"),"",1+SUMPRODUCT(((U$3:U$32&gt;U7)+((U$3:U$32=U7)*(ROW(U$3:U$32)&lt;ROW())))*(T$3:T$32&lt;&gt;"Y")*(B$3:B$32&lt;&gt;"")))</f>
         <v/>
       </c>
       <c r="W7" s="6" t="inlineStr">
@@ -2601,7 +2601,7 @@
         <v/>
       </c>
       <c r="V8" s="9">
-        <f>IF(OR(B8="",T8="Y"),"",1+SUMPRODUCT(((U$3:U$32&gt;U8)+((U$3:U$32=U8)*(ROW(U$3:U$32)&lt;8)))*(T$3:T$32&lt;&gt;"Y")*(B$3:B$32&lt;&gt;"")))</f>
+        <f>IF(OR(B8="",T8="Y"),"",1+SUMPRODUCT(((U$3:U$32&gt;U8)+((U$3:U$32=U8)*(ROW(U$3:U$32)&lt;ROW())))*(T$3:T$32&lt;&gt;"Y")*(B$3:B$32&lt;&gt;"")))</f>
         <v/>
       </c>
       <c r="W8" s="6" t="inlineStr">
@@ -2702,7 +2702,7 @@
         <v/>
       </c>
       <c r="V9" s="9">
-        <f>IF(OR(B9="",T9="Y"),"",1+SUMPRODUCT(((U$3:U$32&gt;U9)+((U$3:U$32=U9)*(ROW(U$3:U$32)&lt;9)))*(T$3:T$32&lt;&gt;"Y")*(B$3:B$32&lt;&gt;"")))</f>
+        <f>IF(OR(B9="",T9="Y"),"",1+SUMPRODUCT(((U$3:U$32&gt;U9)+((U$3:U$32=U9)*(ROW(U$3:U$32)&lt;ROW())))*(T$3:T$32&lt;&gt;"Y")*(B$3:B$32&lt;&gt;"")))</f>
         <v/>
       </c>
       <c r="W9" s="6" t="inlineStr">
@@ -2805,7 +2805,7 @@
         <v/>
       </c>
       <c r="V10" s="9">
-        <f>IF(OR(B10="",T10="Y"),"",1+SUMPRODUCT(((U$3:U$32&gt;U10)+((U$3:U$32=U10)*(ROW(U$3:U$32)&lt;10)))*(T$3:T$32&lt;&gt;"Y")*(B$3:B$32&lt;&gt;"")))</f>
+        <f>IF(OR(B10="",T10="Y"),"",1+SUMPRODUCT(((U$3:U$32&gt;U10)+((U$3:U$32=U10)*(ROW(U$3:U$32)&lt;ROW())))*(T$3:T$32&lt;&gt;"Y")*(B$3:B$32&lt;&gt;"")))</f>
         <v/>
       </c>
       <c r="W10" s="6" t="inlineStr">
@@ -2906,7 +2906,7 @@
         <v/>
       </c>
       <c r="V11" s="9">
-        <f>IF(OR(B11="",T11="Y"),"",1+SUMPRODUCT(((U$3:U$32&gt;U11)+((U$3:U$32=U11)*(ROW(U$3:U$32)&lt;11)))*(T$3:T$32&lt;&gt;"Y")*(B$3:B$32&lt;&gt;"")))</f>
+        <f>IF(OR(B11="",T11="Y"),"",1+SUMPRODUCT(((U$3:U$32&gt;U11)+((U$3:U$32=U11)*(ROW(U$3:U$32)&lt;ROW())))*(T$3:T$32&lt;&gt;"Y")*(B$3:B$32&lt;&gt;"")))</f>
         <v/>
       </c>
       <c r="W11" s="6" t="inlineStr">
@@ -3007,7 +3007,7 @@
         <v/>
       </c>
       <c r="V12" s="9">
-        <f>IF(OR(B12="",T12="Y"),"",1+SUMPRODUCT(((U$3:U$32&gt;U12)+((U$3:U$32=U12)*(ROW(U$3:U$32)&lt;12)))*(T$3:T$32&lt;&gt;"Y")*(B$3:B$32&lt;&gt;"")))</f>
+        <f>IF(OR(B12="",T12="Y"),"",1+SUMPRODUCT(((U$3:U$32&gt;U12)+((U$3:U$32=U12)*(ROW(U$3:U$32)&lt;ROW())))*(T$3:T$32&lt;&gt;"Y")*(B$3:B$32&lt;&gt;"")))</f>
         <v/>
       </c>
       <c r="W12" s="6" t="inlineStr">
@@ -3110,7 +3110,7 @@
         <v/>
       </c>
       <c r="V13" s="9">
-        <f>IF(OR(B13="",T13="Y"),"",1+SUMPRODUCT(((U$3:U$32&gt;U13)+((U$3:U$32=U13)*(ROW(U$3:U$32)&lt;13)))*(T$3:T$32&lt;&gt;"Y")*(B$3:B$32&lt;&gt;"")))</f>
+        <f>IF(OR(B13="",T13="Y"),"",1+SUMPRODUCT(((U$3:U$32&gt;U13)+((U$3:U$32=U13)*(ROW(U$3:U$32)&lt;ROW())))*(T$3:T$32&lt;&gt;"Y")*(B$3:B$32&lt;&gt;"")))</f>
         <v/>
       </c>
       <c r="W13" s="6" t="inlineStr">
@@ -3213,7 +3213,7 @@
         <v/>
       </c>
       <c r="V14" s="9">
-        <f>IF(OR(B14="",T14="Y"),"",1+SUMPRODUCT(((U$3:U$32&gt;U14)+((U$3:U$32=U14)*(ROW(U$3:U$32)&lt;14)))*(T$3:T$32&lt;&gt;"Y")*(B$3:B$32&lt;&gt;"")))</f>
+        <f>IF(OR(B14="",T14="Y"),"",1+SUMPRODUCT(((U$3:U$32&gt;U14)+((U$3:U$32=U14)*(ROW(U$3:U$32)&lt;ROW())))*(T$3:T$32&lt;&gt;"Y")*(B$3:B$32&lt;&gt;"")))</f>
         <v/>
       </c>
       <c r="W14" s="6" t="inlineStr">
@@ -3316,7 +3316,7 @@
         <v/>
       </c>
       <c r="V15" s="9">
-        <f>IF(OR(B15="",T15="Y"),"",1+SUMPRODUCT(((U$3:U$32&gt;U15)+((U$3:U$32=U15)*(ROW(U$3:U$32)&lt;15)))*(T$3:T$32&lt;&gt;"Y")*(B$3:B$32&lt;&gt;"")))</f>
+        <f>IF(OR(B15="",T15="Y"),"",1+SUMPRODUCT(((U$3:U$32&gt;U15)+((U$3:U$32=U15)*(ROW(U$3:U$32)&lt;ROW())))*(T$3:T$32&lt;&gt;"Y")*(B$3:B$32&lt;&gt;"")))</f>
         <v/>
       </c>
       <c r="W15" s="6" t="inlineStr">
@@ -3419,7 +3419,7 @@
         <v/>
       </c>
       <c r="V16" s="9">
-        <f>IF(OR(B16="",T16="Y"),"",1+SUMPRODUCT(((U$3:U$32&gt;U16)+((U$3:U$32=U16)*(ROW(U$3:U$32)&lt;16)))*(T$3:T$32&lt;&gt;"Y")*(B$3:B$32&lt;&gt;"")))</f>
+        <f>IF(OR(B16="",T16="Y"),"",1+SUMPRODUCT(((U$3:U$32&gt;U16)+((U$3:U$32=U16)*(ROW(U$3:U$32)&lt;ROW())))*(T$3:T$32&lt;&gt;"Y")*(B$3:B$32&lt;&gt;"")))</f>
         <v/>
       </c>
       <c r="W16" s="6" t="inlineStr">
@@ -3520,7 +3520,7 @@
         <v/>
       </c>
       <c r="V17" s="9">
-        <f>IF(OR(B17="",T17="Y"),"",1+SUMPRODUCT(((U$3:U$32&gt;U17)+((U$3:U$32=U17)*(ROW(U$3:U$32)&lt;17)))*(T$3:T$32&lt;&gt;"Y")*(B$3:B$32&lt;&gt;"")))</f>
+        <f>IF(OR(B17="",T17="Y"),"",1+SUMPRODUCT(((U$3:U$32&gt;U17)+((U$3:U$32=U17)*(ROW(U$3:U$32)&lt;ROW())))*(T$3:T$32&lt;&gt;"Y")*(B$3:B$32&lt;&gt;"")))</f>
         <v/>
       </c>
       <c r="W17" s="6" t="inlineStr">
@@ -3623,7 +3623,7 @@
         <v/>
       </c>
       <c r="V18" s="9">
-        <f>IF(OR(B18="",T18="Y"),"",1+SUMPRODUCT(((U$3:U$32&gt;U18)+((U$3:U$32=U18)*(ROW(U$3:U$32)&lt;18)))*(T$3:T$32&lt;&gt;"Y")*(B$3:B$32&lt;&gt;"")))</f>
+        <f>IF(OR(B18="",T18="Y"),"",1+SUMPRODUCT(((U$3:U$32&gt;U18)+((U$3:U$32=U18)*(ROW(U$3:U$32)&lt;ROW())))*(T$3:T$32&lt;&gt;"Y")*(B$3:B$32&lt;&gt;"")))</f>
         <v/>
       </c>
       <c r="W18" s="6" t="inlineStr">
@@ -3726,7 +3726,7 @@
         <v/>
       </c>
       <c r="V19" s="9">
-        <f>IF(OR(B19="",T19="Y"),"",1+SUMPRODUCT(((U$3:U$32&gt;U19)+((U$3:U$32=U19)*(ROW(U$3:U$32)&lt;19)))*(T$3:T$32&lt;&gt;"Y")*(B$3:B$32&lt;&gt;"")))</f>
+        <f>IF(OR(B19="",T19="Y"),"",1+SUMPRODUCT(((U$3:U$32&gt;U19)+((U$3:U$32=U19)*(ROW(U$3:U$32)&lt;ROW())))*(T$3:T$32&lt;&gt;"Y")*(B$3:B$32&lt;&gt;"")))</f>
         <v/>
       </c>
       <c r="W19" s="6" t="inlineStr">
@@ -3827,7 +3827,7 @@
         <v/>
       </c>
       <c r="V20" s="9">
-        <f>IF(OR(B20="",T20="Y"),"",1+SUMPRODUCT(((U$3:U$32&gt;U20)+((U$3:U$32=U20)*(ROW(U$3:U$32)&lt;20)))*(T$3:T$32&lt;&gt;"Y")*(B$3:B$32&lt;&gt;"")))</f>
+        <f>IF(OR(B20="",T20="Y"),"",1+SUMPRODUCT(((U$3:U$32&gt;U20)+((U$3:U$32=U20)*(ROW(U$3:U$32)&lt;ROW())))*(T$3:T$32&lt;&gt;"Y")*(B$3:B$32&lt;&gt;"")))</f>
         <v/>
       </c>
       <c r="W20" s="6" t="inlineStr">
@@ -3928,7 +3928,7 @@
         <v/>
       </c>
       <c r="V21" s="9">
-        <f>IF(OR(B21="",T21="Y"),"",1+SUMPRODUCT(((U$3:U$32&gt;U21)+((U$3:U$32=U21)*(ROW(U$3:U$32)&lt;21)))*(T$3:T$32&lt;&gt;"Y")*(B$3:B$32&lt;&gt;"")))</f>
+        <f>IF(OR(B21="",T21="Y"),"",1+SUMPRODUCT(((U$3:U$32&gt;U21)+((U$3:U$32=U21)*(ROW(U$3:U$32)&lt;ROW())))*(T$3:T$32&lt;&gt;"Y")*(B$3:B$32&lt;&gt;"")))</f>
         <v/>
       </c>
       <c r="W21" s="6" t="inlineStr">
@@ -4029,7 +4029,7 @@
         <v/>
       </c>
       <c r="V22" s="9">
-        <f>IF(OR(B22="",T22="Y"),"",1+SUMPRODUCT(((U$3:U$32&gt;U22)+((U$3:U$32=U22)*(ROW(U$3:U$32)&lt;22)))*(T$3:T$32&lt;&gt;"Y")*(B$3:B$32&lt;&gt;"")))</f>
+        <f>IF(OR(B22="",T22="Y"),"",1+SUMPRODUCT(((U$3:U$32&gt;U22)+((U$3:U$32=U22)*(ROW(U$3:U$32)&lt;ROW())))*(T$3:T$32&lt;&gt;"Y")*(B$3:B$32&lt;&gt;"")))</f>
         <v/>
       </c>
       <c r="W22" s="6" t="inlineStr">
@@ -4130,7 +4130,7 @@
         <v/>
       </c>
       <c r="V23" s="9">
-        <f>IF(OR(B23="",T23="Y"),"",1+SUMPRODUCT(((U$3:U$32&gt;U23)+((U$3:U$32=U23)*(ROW(U$3:U$32)&lt;23)))*(T$3:T$32&lt;&gt;"Y")*(B$3:B$32&lt;&gt;"")))</f>
+        <f>IF(OR(B23="",T23="Y"),"",1+SUMPRODUCT(((U$3:U$32&gt;U23)+((U$3:U$32=U23)*(ROW(U$3:U$32)&lt;ROW())))*(T$3:T$32&lt;&gt;"Y")*(B$3:B$32&lt;&gt;"")))</f>
         <v/>
       </c>
       <c r="W23" s="6" t="inlineStr">
@@ -4231,7 +4231,7 @@
         <v/>
       </c>
       <c r="V24" s="9">
-        <f>IF(OR(B24="",T24="Y"),"",1+SUMPRODUCT(((U$3:U$32&gt;U24)+((U$3:U$32=U24)*(ROW(U$3:U$32)&lt;24)))*(T$3:T$32&lt;&gt;"Y")*(B$3:B$32&lt;&gt;"")))</f>
+        <f>IF(OR(B24="",T24="Y"),"",1+SUMPRODUCT(((U$3:U$32&gt;U24)+((U$3:U$32=U24)*(ROW(U$3:U$32)&lt;ROW())))*(T$3:T$32&lt;&gt;"Y")*(B$3:B$32&lt;&gt;"")))</f>
         <v/>
       </c>
       <c r="W24" s="6" t="inlineStr">
@@ -4334,7 +4334,7 @@
         <v/>
       </c>
       <c r="V25" s="9">
-        <f>IF(OR(B25="",T25="Y"),"",1+SUMPRODUCT(((U$3:U$32&gt;U25)+((U$3:U$32=U25)*(ROW(U$3:U$32)&lt;25)))*(T$3:T$32&lt;&gt;"Y")*(B$3:B$32&lt;&gt;"")))</f>
+        <f>IF(OR(B25="",T25="Y"),"",1+SUMPRODUCT(((U$3:U$32&gt;U25)+((U$3:U$32=U25)*(ROW(U$3:U$32)&lt;ROW())))*(T$3:T$32&lt;&gt;"Y")*(B$3:B$32&lt;&gt;"")))</f>
         <v/>
       </c>
       <c r="W25" s="6" t="inlineStr">
@@ -4435,7 +4435,7 @@
         <v/>
       </c>
       <c r="V26" s="9">
-        <f>IF(OR(B26="",T26="Y"),"",1+SUMPRODUCT(((U$3:U$32&gt;U26)+((U$3:U$32=U26)*(ROW(U$3:U$32)&lt;26)))*(T$3:T$32&lt;&gt;"Y")*(B$3:B$32&lt;&gt;"")))</f>
+        <f>IF(OR(B26="",T26="Y"),"",1+SUMPRODUCT(((U$3:U$32&gt;U26)+((U$3:U$32=U26)*(ROW(U$3:U$32)&lt;ROW())))*(T$3:T$32&lt;&gt;"Y")*(B$3:B$32&lt;&gt;"")))</f>
         <v/>
       </c>
       <c r="W26" s="6" t="inlineStr">
@@ -4536,7 +4536,7 @@
         <v/>
       </c>
       <c r="V27" s="9">
-        <f>IF(OR(B27="",T27="Y"),"",1+SUMPRODUCT(((U$3:U$32&gt;U27)+((U$3:U$32=U27)*(ROW(U$3:U$32)&lt;27)))*(T$3:T$32&lt;&gt;"Y")*(B$3:B$32&lt;&gt;"")))</f>
+        <f>IF(OR(B27="",T27="Y"),"",1+SUMPRODUCT(((U$3:U$32&gt;U27)+((U$3:U$32=U27)*(ROW(U$3:U$32)&lt;ROW())))*(T$3:T$32&lt;&gt;"Y")*(B$3:B$32&lt;&gt;"")))</f>
         <v/>
       </c>
       <c r="W27" s="6" t="inlineStr">
@@ -4639,7 +4639,7 @@
         <v/>
       </c>
       <c r="V28" s="9">
-        <f>IF(OR(B28="",T28="Y"),"",1+SUMPRODUCT(((U$3:U$32&gt;U28)+((U$3:U$32=U28)*(ROW(U$3:U$32)&lt;28)))*(T$3:T$32&lt;&gt;"Y")*(B$3:B$32&lt;&gt;"")))</f>
+        <f>IF(OR(B28="",T28="Y"),"",1+SUMPRODUCT(((U$3:U$32&gt;U28)+((U$3:U$32=U28)*(ROW(U$3:U$32)&lt;ROW())))*(T$3:T$32&lt;&gt;"Y")*(B$3:B$32&lt;&gt;"")))</f>
         <v/>
       </c>
       <c r="W28" s="6" t="inlineStr">
@@ -4736,7 +4736,7 @@
         <v/>
       </c>
       <c r="V29" s="9">
-        <f>IF(OR(B29="",T29="Y"),"",1+SUMPRODUCT(((U$3:U$32&gt;U29)+((U$3:U$32=U29)*(ROW(U$3:U$32)&lt;29)))*(T$3:T$32&lt;&gt;"Y")*(B$3:B$32&lt;&gt;"")))</f>
+        <f>IF(OR(B29="",T29="Y"),"",1+SUMPRODUCT(((U$3:U$32&gt;U29)+((U$3:U$32=U29)*(ROW(U$3:U$32)&lt;ROW())))*(T$3:T$32&lt;&gt;"Y")*(B$3:B$32&lt;&gt;"")))</f>
         <v/>
       </c>
       <c r="W29" s="6" t="inlineStr">
@@ -4837,7 +4837,7 @@
         <v/>
       </c>
       <c r="V30" s="9">
-        <f>IF(OR(B30="",T30="Y"),"",1+SUMPRODUCT(((U$3:U$32&gt;U30)+((U$3:U$32=U30)*(ROW(U$3:U$32)&lt;30)))*(T$3:T$32&lt;&gt;"Y")*(B$3:B$32&lt;&gt;"")))</f>
+        <f>IF(OR(B30="",T30="Y"),"",1+SUMPRODUCT(((U$3:U$32&gt;U30)+((U$3:U$32=U30)*(ROW(U$3:U$32)&lt;ROW())))*(T$3:T$32&lt;&gt;"Y")*(B$3:B$32&lt;&gt;"")))</f>
         <v/>
       </c>
       <c r="W30" s="6" t="inlineStr">
@@ -4940,7 +4940,7 @@
         <v/>
       </c>
       <c r="V31" s="9">
-        <f>IF(OR(B31="",T31="Y"),"",1+SUMPRODUCT(((U$3:U$32&gt;U31)+((U$3:U$32=U31)*(ROW(U$3:U$32)&lt;31)))*(T$3:T$32&lt;&gt;"Y")*(B$3:B$32&lt;&gt;"")))</f>
+        <f>IF(OR(B31="",T31="Y"),"",1+SUMPRODUCT(((U$3:U$32&gt;U31)+((U$3:U$32=U31)*(ROW(U$3:U$32)&lt;ROW())))*(T$3:T$32&lt;&gt;"Y")*(B$3:B$32&lt;&gt;"")))</f>
         <v/>
       </c>
       <c r="W31" s="6" t="inlineStr">
@@ -5041,7 +5041,7 @@
         <v/>
       </c>
       <c r="V32" s="9">
-        <f>IF(OR(B32="",T32="Y"),"",1+SUMPRODUCT(((U$3:U$32&gt;U32)+((U$3:U$32=U32)*(ROW(U$3:U$32)&lt;32)))*(T$3:T$32&lt;&gt;"Y")*(B$3:B$32&lt;&gt;"")))</f>
+        <f>IF(OR(B32="",T32="Y"),"",1+SUMPRODUCT(((U$3:U$32&gt;U32)+((U$3:U$32=U32)*(ROW(U$3:U$32)&lt;ROW())))*(T$3:T$32&lt;&gt;"Y")*(B$3:B$32&lt;&gt;"")))</f>
         <v/>
       </c>
       <c r="W32" s="6" t="inlineStr">

</xml_diff>